<commit_message>
scenario engine: invite links, ty/vy, scheduler, surveys, demo /next
</commit_message>
<xml_diff>
--- a/scenario/scenario.xlsx
+++ b/scenario/scenario.xlsx
@@ -1661,18 +1661,22 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Хорошо! Если передумаешь, напиши /food — пришлю список. Или просто спроси меня, где поесть.</t>
+          <t>Хорошо! Если передумаешь, просто спроси меня, где поесть.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Хорошо! Если передумаете, напишите /food — пришлю список. Или просто спросите меня, где поесть.</t>
+          <t>Хорошо! Если передумаете, просто спросите меня, где поесть.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Правка движка: убрали /food, такой команды в боте нет, про еду новичок спрашивает своими словами.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2025,13 +2029,13 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>{имя}, давай я представлю тебя коллегам. Напиши пару строк о себе: опыт, сильные стороны, увлечения. Если хочешь, пришли фото. Я соберу из этого короткое знакомство и покажу тебе перед публикацией.
+          <t>{имя}, давай я представлю тебя коллегам. Напиши пару строк о себе: опыт, сильные стороны, увлечения. Я передам это коллегам из HR, они подготовят короткое знакомство.
 Пример: «Знакомьтесь, это Анна, наш новый инженер-технолог. Пять лет работала на производстве полимерных труб. В свободное время бегает и собирает настольные игры».</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>{имя}, давайте я представлю вас коллегам. Напишите пару строк о себе: опыт, сильные стороны, увлечения. Если хотите, пришлите фото. Я соберу из этого короткое знакомство и покажу вам перед публикацией.
+          <t>{имя}, давайте я представлю вас коллегам. Напишите пару строк о себе: опыт, сильные стороны, увлечения. Я передам это коллегам из HR, они подготовят короткое знакомство.
 Пример: «Знакомьтесь, это Анна, наш новый инженер-технолог. Пять лет работала на производстве полимерных труб. В свободное время бегает и собирает настольные игры».</t>
         </is>
       </c>
@@ -2040,7 +2044,8 @@
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Было «Составь, пожалуйста, краткое описание… (образец)» — звучало как задание. Объяснили зачем, фото — по желанию, добавили образец и согласование перед публикацией. Черновик знакомства собирает ИИ из ответа новичка. В исходнике «по отмашке рекрутера», сейчас уходит всем. Бот сохраняет ответ, сам знакомство не публикует.</t>
+          <t>Было «Составь, пожалуйста, краткое описание… (образец)» — звучало как задание. Объяснили зачем, фото — по желанию, добавили образец и согласование перед публикацией. Черновик знакомства собирает ИИ из ответа новичка. В исходнике «по отмашке рекрутера», сейчас уходит всем. Бот сохраняет ответ, сам знакомство не публикует.
+Правка движка: бот не принимает фото и не показывает черновик, ответ сохраняется и уходит рекрутеру.</t>
         </is>
       </c>
     </row>
@@ -2101,14 +2106,14 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Чтобы было понятно, к чему двигаться на испытательном сроке, твой руководитель подготовил адаптационный план. Вот он.
+          <t>Чтобы было понятно, к чему двигаться на испытательном сроке, твой руководитель подготовил адаптационный план.
 Если что-то в нём непонятно, спроси руководителя напрямую — это нормально. Или напиши мне.
 [HR: приложить адаптационный план]</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Чтобы было понятно, к чему двигаться на испытательном сроке, ваш руководитель подготовил адаптационный план. Вот он.
+          <t>Чтобы было понятно, к чему двигаться на испытательном сроке, ваш руководитель подготовил адаптационный план.
 Если что-то в нём непонятно, спросите руководителя напрямую — это нормально. Или напишите мне.
 [HR: приложить адаптационный план]</t>
         </is>
@@ -2122,7 +2127,8 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>«Не бойся обращаться» → «это нормально». Убрали «Надеюсь, ты уже чуть лучше понимаешь наши ценности и правила». План бот сам не прикладывает, см. пометку [HR: ...].</t>
+          <t>«Не бойся обращаться» → «это нормально». Убрали «Надеюсь, ты уже чуть лучше понимаешь наши ценности и правила». План бот сам не прикладывает, см. пометку [HR: ...].
+Правка движка: убрали «Вот он.», плана во вложении пока нет.</t>
         </is>
       </c>
     </row>
@@ -3216,18 +3222,22 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Спасибо, что честно говоришь. Напиши, что мешает, — передам в отдел подбора. Или свяжись с HR-специалистом напрямую: команда /hr.</t>
+          <t>Спасибо, что честно говоришь. Напиши, что мешает, — передам в отдел подбора.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Спасибо, что честно говорите. Напишите, что мешает, — передам в отдел подбора. Или свяжитесь с HR-специалистом напрямую: команда /hr.</t>
+          <t>Спасибо, что честно говорите. Напишите, что мешает, — передам в отдел подбора.</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr"/>
-      <c r="K72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>Правка движка: убрали команду /hr, её в боте нет. Ответ новичка бот передаёт сам.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fixes after review: question ids, failed sends, dashes, timeouts
</commit_message>
<xml_diff>
--- a/scenario/scenario.xlsx
+++ b/scenario/scenario.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Здравствуйте! Я Корсик 🐾 — помощник новичков Группы ПОЛИПЛАСТИК.
+          <t>Здравствуйте! Я Корсик 🐾, помощник новичков Группы ПОЛИПЛАСТИК.
 Первые три месяца я буду рядом: подскажу, что взять с собой в первый день, как добраться и к кому идти с вопросами. А если что-то непонятно, можно просто написать мне, как коллеге.</t>
         </is>
       </c>
@@ -566,7 +566,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Как нам удобнее общаться — на «ты» или на «вы»?</t>
+          <t>Как нам удобнее общаться: на «ты» или на «вы»?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
@@ -641,13 +641,13 @@
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Коротко обо мне: я чат-бот, которого сделали, чтобы первые месяцы на новом месте прошли спокойнее.
-До конца испытательного срока буду писать тебе в нужные моменты: что подготовить, что почитать, с кем познакомиться. А в любой момент можно задать мне вопрос — отвечу сам или передам коллегам из HR.</t>
+До конца испытательного срока буду писать тебе в нужные моменты: что подготовить, что почитать, с кем познакомиться. А в любой момент можно задать мне вопрос: отвечу сам или передам коллегам из HR.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Коротко обо мне: я чат-бот, которого сделали, чтобы первые месяцы на новом месте прошли спокойнее.
-До конца испытательного срока буду писать вам в нужные моменты: что подготовить, что почитать, с кем познакомиться. А в любой момент можно задать мне вопрос — отвечу сам или передам коллегам из HR.</t>
+До конца испытательного срока буду писать вам в нужные моменты: что подготовить, что почитать, с кем познакомиться. А в любой момент можно задать мне вопрос: отвечу сам или передам коллегам из HR.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -659,7 +659,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Было два варианта на выбор — объединили в один. Добавили главное: боту можно задавать вопросы в любой момент.</t>
+          <t>Было два варианта на выбор, объединили в один. Добавили главное: боту можно задавать вопросы в любой момент.</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Чтобы оформление в первый день прошло быстро, собери, пожалуйста, документы из списка ниже. Если чего-то не хватает, напиши мне — передам вопрос рекрутеру.
+          <t>Чтобы оформление в первый день прошло быстро, собери, пожалуйста, документы из списка ниже. Если чего-то не хватает, напиши мне, передам вопрос рекрутеру.
 Документы для оформления:
 1. Бумажная трудовая книжка и сведения о трудовой деятельности (их можно выгрузить на Госуслугах).
 2. Паспорт.
@@ -701,7 +701,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Чтобы оформление в первый день прошло быстро, соберите, пожалуйста, документы из списка ниже. Если чего-то не хватает, напишите мне — передам вопрос рекрутеру.
+          <t>Чтобы оформление в первый день прошло быстро, соберите, пожалуйста, документы из списка ниже. Если чего-то не хватает, напишите мне, передам вопрос рекрутеру.
 Документы для оформления:
 1. Бумажная трудовая книжка и сведения о трудовой деятельности (их можно выгрузить на Госуслугах).
 2. Паспорт.
@@ -722,7 +722,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Было «чтобы ты пришел подготовленный» — мужской род и канцелярит. Добавили, что делать, если документа нет. Список в колонке J — без «Вашего», с единым оформлением. Список документов из колонки J добавлен в конец текста.</t>
+          <t>Было «чтобы ты пришел подготовленный»: мужской род и канцелярит. Добавили, что делать, если документа нет. Список в колонке J: без «Вашего», с единым оформлением. Список документов из колонки J добавлен в конец текста.</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Чтобы оформление в первый день прошло быстро, собери, пожалуйста, документы из списка ниже. Если чего-то не хватает, напиши мне — передам вопрос рекрутеру.
+          <t>Чтобы оформление в первый день прошло быстро, собери, пожалуйста, документы из списка ниже. Если чего-то не хватает, напиши мне, передам вопрос рекрутеру.
 Документы для оформления:
 1. Бумажная трудовая книжка и сведения о трудовой деятельности (их можно выгрузить на Госуслугах).
 2. Паспорт.
@@ -765,7 +765,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Чтобы оформление в первый день прошло быстро, соберите, пожалуйста, документы из списка ниже. Если чего-то не хватает, напишите мне — передам вопрос рекрутеру.
+          <t>Чтобы оформление в первый день прошло быстро, соберите, пожалуйста, документы из списка ниже. Если чего-то не хватает, напишите мне, передам вопрос рекрутеру.
 Документы для оформления:
 1. Бумажная трудовая книжка и сведения о трудовой деятельности (их можно выгрузить на Госуслугах).
 2. Паспорт.
@@ -787,7 +787,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Как в строке 9. Для GTP в списке есть фото 3×4, для GrPP и Luzhniki — нет. Уточнить у HR, так и задумано или фото нужно всем. Список документов из колонки J добавлен в конец текста.</t>
+          <t>Как в строке 9. Для GTP в списке есть фото 3×4, для GrPP и Luzhniki - нет. Уточнить у HR, так и задумано или фото нужно всем. Список документов из колонки J добавлен в конец текста.</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Пока есть время до первого дня — немного о компании, в которую ты приходишь.
+          <t>Пока есть время до первого дня, немного о компании, в которую ты приходишь.
 🏭 Группе ПОЛИПЛАСТИК 35 лет, в команде около 8500 человек.
 💧 Мы делаем трубопроводные системы и решения для очистки сточных вод, а ещё композиционные материалы из термопластов. Наши трубы работают в коммунальной, промышленной и аграрной инфраструктуре.
 💡 Здесь ценят инициативу: если есть идея, её можно и нужно предлагать.
@@ -931,7 +931,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Пока есть время до первого дня — немного о компании, в которую вы приходите.
+          <t>Пока есть время до первого дня, немного о компании, в которую вы приходите.
 🏭 Группе ПОЛИПЛАСТИК 35 лет, в команде около 8500 человек.
 💧 Мы делаем трубопроводные системы и решения для очистки сточных вод, а ещё композиционные материалы из термопластов. Наши трубы работают в коммунальной, промышленной и аграрной инфраструктуре.
 💡 Здесь ценят инициативу: если есть идея, её можно и нужно предлагать.
@@ -967,13 +967,13 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>На этом пока всё — отдыхай перед стартом. Напишу за день до выхода.
+          <t>На этом пока всё, отдыхай перед стартом. Напишу за день до выхода.
 До встречи, {имя}! 👋</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>На этом пока всё — отдохните перед стартом. Напишу за день до выхода.
+          <t>На этом пока всё, отдохните перед стартом. Напишу за день до выхода.
 До встречи, {имя}! 👋</t>
         </is>
       </c>
@@ -1023,7 +1023,7 @@
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Кнопка «Готов/Готова» → «Всё готово», без рода. Убрали шутку «я сам через это проходил, когда меня создавали» — она обесценивает волнение. Добавили, что боту можно писать. Время в исходнике не указано, взяли 10:00. Ответ сохраняется как опрос.</t>
+          <t>Кнопка «Готов/Готова» → «Всё готово», без рода. Убрали шутку «я сам через это проходил, когда меня создавали»: она обесценивает волнение. Добавили, что боту можно писать. Время в исходнике не указано, взяли 10:00. Ответ сохраняется как опрос.</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Это нормально, перед первым днём волнуются почти все. Завтра я весь день на связи — на любой вопрос можно просто написать мне.</t>
+          <t>Это нормально, перед первым днём волнуются почти все. Завтра я весь день на связи: на любой вопрос можно просто написать мне.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Напоминаю про документы для оформления — список ниже. Возьми их, пожалуйста, завтра с собой.
+          <t>Напоминаю про документы для оформления: список ниже. Возьми их, пожалуйста, завтра с собой.
 Документы для оформления:
 1. Бумажная трудовая книжка и сведения о трудовой деятельности (их можно выгрузить на Госуслугах).
 2. Паспорт.
@@ -1182,7 +1182,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Напоминаю про документы для оформления — список ниже. Возьмите их, пожалуйста, завтра с собой.
+          <t>Напоминаю про документы для оформления: список ниже. Возьмите их, пожалуйста, завтра с собой.
 Документы для оформления:
 1. Бумажная трудовая книжка и сведения о трудовой деятельности (их можно выгрузить на Госуслугах).
 2. Паспорт.
@@ -1204,7 +1204,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Короче. Текст из колонки D («Напомнить кандидату о списке документов…») перенесли в колонку C: это информационный повод, а не тег сотрудника. Тег пустой — значит, для всех площадок. Список документов из колонки J добавлен в конец текста.</t>
+          <t>Короче. Текст из колонки D («Напомнить кандидату о списке документов…») перенесли в колонку C: это информационный повод, а не тег сотрудника. Тег пустой - значит, для всех площадок. Список документов из колонки J добавлен в конец текста.</t>
         </is>
       </c>
     </row>
@@ -1229,13 +1229,13 @@
       <c r="F19" s="2" t="inlineStr">
         <is>
           <t>{имя}, с первым рабочим днём! 🎉
-Сегодня будет много нового: люди, места, системы. Не стесняйся спрашивать — у коллег, у руководителя или у меня. Здесь все когда-то были новичками.</t>
+Сегодня будет много нового: люди, места, системы. Не стесняйся спрашивать: у коллег, у руководителя или у меня. Здесь все когда-то были новичками.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>{имя}, с первым рабочим днём! 🎉
-Сегодня будет много нового: люди, места, системы. Не стесняйтесь спрашивать — у коллег, у руководителя или у меня. Здесь все когда-то были новичками.</t>
+Сегодня будет много нового: люди, места, системы. Не стесняйтесь спрашивать: у коллег, у руководителя или у меня. Здесь все когда-то были новичками.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -1431,12 +1431,12 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>В первый день такое бывает. Напиши, чего именно нет, — передам рекрутеру. А сроки лучше уточнить у руководителя: он знает, когда всё будет готово.</t>
+          <t>В первый день такое бывает. Напиши, чего именно нет, передам рекрутеру. А сроки лучше уточнить у руководителя: он знает, когда всё будет готово.</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>В первый день такое бывает. Напишите, чего именно нет, — передам рекрутеру. А сроки лучше уточнить у руководителя: он знает, когда всё будет готово.</t>
+          <t>В первый день такое бывает. Напишите, чего именно нет, передам рекрутеру. А сроки лучше уточнить у руководителя: он знает, когда всё будет готово.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -1550,12 +1550,12 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>В первый день такое бывает. Напиши, чего именно нет, — передам рекрутеру. А сроки лучше уточнить у руководителя: он знает, когда всё будет готово.</t>
+          <t>В первый день такое бывает. Напиши, чего именно нет, передам рекрутеру. А сроки лучше уточнить у руководителя: он знает, когда всё будет готово.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>В первый день такое бывает. Напишите, чего именно нет, — передам рекрутеру. А сроки лучше уточнить у руководителя: он знает, когда всё будет готово.</t>
+          <t>В первый день такое бывает. Напишите, чего именно нет, передам рекрутеру. А сроки лучше уточнить у руководителя: он знает, когда всё будет готово.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Было «Дарю небольшую открытку!». Служебные пометки для бота — в квадратных скобках.</t>
+          <t>Было «Дарю небольшую открытку!». Служебные пометки для бота - в квадратных скобках.</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Команда /Food → /food (строчными, как принято для команд). Добавили, что можно спросить своими словами — это понимает ИИ-модуль. Кнопка «Да, подскажи» стала «Да!»: колонка кнопок общая для «ты» и «вы». Команды /food в боте пока нет, работает вопрос своими словами.</t>
+          <t>Команда /Food → /food (строчными, как принято для команд). Добавили, что можно спросить своими словами: это понимает ИИ-модуль. Кнопка «Да, подскажи» стала «Да!»: колонка кнопок общая для «ты» и «вы». Команды /food в боте пока нет, работает вопрос своими словами.</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Без «ты/вы». Пометка про вложение — в скобках. PDF бот не отправляет, только картинки: список лучше вписать текстом.</t>
+          <t>Без «ты/вы». Пометка про вложение - в скобках. PDF бот не отправляет, только картинки: список лучше вписать текстом.</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Было «ты уже немного освоился» — мужской род. Сократили.</t>
+          <t>Было «ты уже немного освоился»: мужской род. Сократили.</t>
         </is>
       </c>
     </row>
@@ -1862,7 +1862,7 @@
       <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Вот справочник с контактами коллег: https://my.polyplastic.ru/employees/Pages/address-book.aspx
-Он открывается только с рабочего компьютера в корпоративной сети или под корпоративной учётной записью — с личного телефона не откроется.</t>
+Он открывается только с рабочего компьютера в корпоративной сети или под корпоративной учётной записью: с личного телефона не откроется.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
@@ -1908,7 +1908,7 @@
       <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Вот справочник с контактами коллег: http://ats/
-Он открывается только с рабочего компьютера в корпоративной сети или под корпоративной учётной записью — с личного телефона не откроется.</t>
+Он открывается только с рабочего компьютера в корпоративной сети или под корпоративной учётной записью: с личного телефона не откроется.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
@@ -1945,14 +1945,14 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Немного о том, ради чего мы работаем. Наша миссия — «улучшать качество жизни людей, создавая удобную и долговечную инфраструктуру для жизни и бизнеса, развивая новый технологический уклад, задавая отраслевые стандарты качества продукта и сервиса».
+          <t>Немного о том, ради чего мы работаем. Наша миссия: «улучшать качество жизни людей, создавая удобную и долговечную инфраструктуру для жизни и бизнеса, развивая новый технологический уклад, задавая отраслевые стандарты качества продукта и сервиса».
 Теперь ты тоже часть этой команды, и от твоей работы это зависит.
 [HR: приложить корпоративную презентацию]</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Немного о том, ради чего мы работаем. Наша миссия — «улучшать качество жизни людей, создавая удобную и долговечную инфраструктуру для жизни и бизнеса, развивая новый технологический уклад, задавая отраслевые стандарты качества продукта и сервиса».
+          <t>Немного о том, ради чего мы работаем. Наша миссия: «улучшать качество жизни людей, создавая удобную и долговечную инфраструктуру для жизни и бизнеса, развивая новый технологический уклад, задавая отраслевые стандарты качества продукта и сервиса».
 Теперь вы тоже часть этой команды, и от вашей работы это зависит.
 [HR: приложить корпоративную презентацию]</t>
         </is>
@@ -1962,7 +1962,7 @@
       <c r="J37" s="2" t="inlineStr"/>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Миссию оставили дословно — это официальная формулировка. Убрали «Мы ценим каждого сотрудника и верим, что только вместе…»: общие слова, которые есть в любом приветствии.</t>
+          <t>Миссию оставили дословно: это официальная формулировка. Убрали «Мы ценим каждого сотрудника и верим, что только вместе…»: общие слова, которые есть в любом приветствии.</t>
         </is>
       </c>
     </row>
@@ -1987,13 +1987,13 @@
       <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Первый рабочий день позади! Как прошло?
-Если остались вопросы — пиши, разберёмся. А сейчас отдыхай, завтра продолжим.</t>
+Если остались вопросы, пиши, разберёмся. А сейчас отдыхай, завтра продолжим.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Первый рабочий день позади! Как прошло?
-Если остались вопросы — пишите, разберёмся. А сейчас отдыхайте, завтра продолжим.</t>
+Если остались вопросы, пишите, разберёмся. А сейчас отдыхайте, завтра продолжим.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Убрали «я уверен, что ты успешно справился»: мужской род, и бот не знает, как прошёл день. Добавили открытый вопрос — ответ разберёт ИИ-модуль настроений. В исходнике «для сотрудников офиса», тега не было: если нужно, поставить тег.</t>
+          <t>Убрали «я уверен, что ты успешно справился»: мужской род, и бот не знает, как прошёл день. Добавили открытый вопрос: ответ разберёт ИИ-модуль настроений. В исходнике «для сотрудников офиса», тега не было: если нужно, поставить тег.</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Было «Составь, пожалуйста, краткое описание… (образец)» — звучало как задание. Объяснили зачем, фото — по желанию, добавили образец и согласование перед публикацией. Черновик знакомства собирает ИИ из ответа новичка. В исходнике «по отмашке рекрутера», сейчас уходит всем. Бот сохраняет ответ, сам знакомство не публикует.
+          <t>Было «Составь, пожалуйста, краткое описание… (образец)»: звучало как задание. Объяснили зачем, фото - по желанию, добавили образец и согласование перед публикацией. Черновик знакомства собирает ИИ из ответа новичка. В исходнике «по отмашке рекрутера», сейчас уходит всем. Бот сохраняет ответ, сам знакомство не публикует.
 Правка движка: бот не принимает фото и не показывает черновик, ответ сохраняется и уходит рекрутеру.</t>
         </is>
       </c>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Привет, {имя}! Уже третий день — время летит.</t>
+          <t>Привет, {имя}! Уже третий день, время летит.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Здравствуйте, {имя}! Уже третий день — время летит.</t>
+          <t>Здравствуйте, {имя}! Уже третий день, время летит.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -2107,14 +2107,14 @@
       <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Чтобы было понятно, к чему двигаться на испытательном сроке, твой руководитель подготовил адаптационный план.
-Если что-то в нём непонятно, спроси руководителя напрямую — это нормально. Или напиши мне.
+Если что-то в нём непонятно, спроси руководителя напрямую, это нормально. Или напиши мне.
 [HR: приложить адаптационный план]</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
           <t>Чтобы было понятно, к чему двигаться на испытательном сроке, ваш руководитель подготовил адаптационный план.
-Если что-то в нём непонятно, спросите руководителя напрямую — это нормально. Или напишите мне.
+Если что-то в нём непонятно, спросите руководителя напрямую, это нормально. Или напишите мне.
 [HR: приложить адаптационный план]</t>
         </is>
       </c>
@@ -2189,12 +2189,12 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Первые дни на новом месте обычно самые насыщенные. Ответь, пожалуйста, на три коротких вопроса — это минута, а нам поможет сделать адаптацию лучше.</t>
+          <t>Первые дни на новом месте обычно самые насыщенные. Ответь, пожалуйста, на три коротких вопроса - это минута, а нам поможет сделать адаптацию лучше.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Первые дни на новом месте обычно самые насыщенные. Ответьте, пожалуйста, на три коротких вопроса — это минута, а нам поможет сделать адаптацию лучше.</t>
+          <t>Первые дни на новом месте обычно самые насыщенные. Ответьте, пожалуйста, на три коротких вопроса - это минута, а нам поможет сделать адаптацию лучше.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Понял. Рекрутер на связи — можно написать ему напрямую.</t>
+          <t>Понял. Рекрутер на связи: можно написать ему напрямую.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
@@ -2342,7 +2342,7 @@
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Было «ты вышел на работу в период большой нагрузки» — мужской род. «Не бойся поднять этот вопрос» → «скажи об этом».</t>
+          <t>Было «ты вышел на работу в период большой нагрузки»: мужской род. «Не бойся поднять этот вопрос» → «скажи об этом».</t>
         </is>
       </c>
     </row>
@@ -2366,12 +2366,12 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Жаль, что пока не получилось познакомиться. Возможно, у команды сейчас горячий период — так бывает. Но если кажется, что что-то идёт не так, скажи об этом руководителю или напиши мне — передам коллегам из HR.</t>
+          <t>Жаль, что пока не получилось познакомиться. Возможно, у команды сейчас горячий период, так бывает. Но если кажется, что что-то идёт не так, скажи об этом руководителю или напиши мне, передам коллегам из HR.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Жаль, что пока не получилось познакомиться. Возможно, у команды сейчас горячий период — так бывает. Но если кажется, что что-то идёт не так, скажите об этом руководителю или напишите мне — передам коллегам из HR.</t>
+          <t>Жаль, что пока не получилось познакомиться. Возможно, у команды сейчас горячий период, так бывает. Но если кажется, что что-то идёт не так, скажите об этом руководителю или напишите мне, передам коллегам из HR.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -2498,12 +2498,12 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Понимать свои задачи — главное на испытательном сроке. Лучше сразу поговорить с руководителем о том, что от тебя ждут в ближайшие три месяца. Если после разговора яснее не станет, напиши мне — передам в отдел подбора.</t>
+          <t>Понимать свои задачи - главное на испытательном сроке. Лучше сразу поговорить с руководителем о том, что от тебя ждут в ближайшие три месяца. Если после разговора яснее не станет, напиши мне, передам в отдел подбора.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Понимать свои задачи — главное на испытательном сроке. Лучше сразу поговорить с руководителем о том, что от вас ждут в ближайшие три месяца. Если после разговора яснее не станет, напишите мне — передам в отдел подбора.</t>
+          <t>Понимать свои задачи - главное на испытательном сроке. Лучше сразу поговорить с руководителем о том, что от вас ждут в ближайшие три месяца. Если после разговора яснее не станет, напишите мне, передам в отдел подбора.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -2581,7 +2581,7 @@
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Было «Сегодня я хотел бы рассказать тебе об еще одном аспекте работы в нашей компании» — канцелярит. Время в исходнике не указано, взяли 10:00.</t>
+          <t>Было «Сегодня я хотел бы рассказать тебе об еще одном аспекте работы в нашей компании»: канцелярит. Время в исходнике не указано, взяли 10:00.</t>
         </is>
       </c>
     </row>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Корпоративные праздники у нас — не формальность, а способ узнать друг друга не только по работе. Бывают классические корпоративы, спортивные соревнования, профессиональные и календарные праздники.</t>
+          <t>Корпоративные праздники у нас - не формальность, а способ узнать друг друга не только по работе. Бывают классические корпоративы, спортивные соревнования, профессиональные и календарные праздники.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr"/>
@@ -2663,7 +2663,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Пометка про вложение — в скобках. В исходнике картинка «ФОТО», назвали photo_1.png.</t>
+          <t>Пометка про вложение - в скобках. В исходнике картинка «ФОТО», назвали photo_1.png.</t>
         </is>
       </c>
     </row>
@@ -2728,12 +2728,12 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Привет, {имя}! Две недели позади — как ты? Хочу задать несколько вопросов, чтобы понять, всё ли в порядке и где нужна помощь. Это пара минут.</t>
+          <t>Привет, {имя}! Две недели позади - как ты? Хочу задать несколько вопросов, чтобы понять, всё ли в порядке и где нужна помощь. Это пара минут.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Здравствуйте, {имя}! Две недели позади — как вы? Хочу задать несколько вопросов, чтобы понять, всё ли в порядке и где нужна помощь. Это пара минут.</t>
+          <t>Здравствуйте, {имя}! Две недели позади - как вы? Хочу задать несколько вопросов, чтобы понять, всё ли в порядке и где нужна помощь. Это пара минут.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Вопросы были на «вы» в боте на «ты» — теперь две версии. Шкалы и правило «ниже 8 — уточнить причину» сохранили. В МАКС нет встроенных опросов: шкала 1–10 — это два ряда по 5 кнопок. Предлагаем сократить до 3 главных вопросов с уточнением только там, где оценка низкая (см. описание решения). Девять вопросов разбиты на шаги 47.1-47.9: «да/нет» это опрос, оценки это шкала. При «Нет» или оценке ниже 8 бот спрашивает, что не так.</t>
+          <t>Вопросы были на «вы» в боте на «ты»: теперь две версии. Шкалы и правило «ниже 8 - уточнить причину» сохранили. В МАКС нет встроенных опросов: шкала 1–10 - это два ряда по 5 кнопок. Предлагаем сократить до 3 главных вопросов с уточнением только там, где оценка низкая (см. описание решения). Девять вопросов разбиты на шаги 47.1-47.9: «да/нет» это опрос, оценки это шкала. При «Нет» или оценке ниже 8 бот спрашивает, что не так.</t>
         </is>
       </c>
     </row>
@@ -2769,12 +2769,12 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>1 из 9. Понятны ли тебе задачи? — Да / Нет</t>
+          <t>1 из 9. Понятны ли тебе задачи? - Да / Нет</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>1 из 9. Понятны ли вам задачи? — Да / Нет</t>
+          <t>1 из 9. Понятны ли вам задачи? - Да / Нет</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2 из 9. Хватает ли информации, чтобы хорошо делать свою работу? — Да / Нет</t>
+          <t>2 из 9. Хватает ли информации, чтобы хорошо делать свою работу? - Да / Нет</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
@@ -2847,7 +2847,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>3 из 9. Насколько руководитель доступен для вопросов и обратной связи? — от 1 (недоступен) до 10 (всегда на связи)</t>
+          <t>3 из 9. Насколько руководитель доступен для вопросов и обратной связи? - от 1 (недоступен) до 10 (всегда на связи)</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr"/>
@@ -2880,7 +2880,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>4 из 9. Насколько полезна обратная связь от руководителя? — от 1 (её нет) до 10 (подробная и по делу)</t>
+          <t>4 из 9. Насколько полезна обратная связь от руководителя? - от 1 (её нет) до 10 (подробная и по делу)</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr"/>
@@ -2913,7 +2913,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>5 из 9. Помогают ли коллеги, когда возникают вопросы или сложности? — от 1 (не помогают) до 10 (всегда помогают)</t>
+          <t>5 из 9. Помогают ли коллеги, когда возникают вопросы или сложности? - от 1 (не помогают) до 10 (всегда помогают)</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr"/>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>6 из 9. Как помогли с техникой, доступами и рабочим местом? — от 1 (плохо) до 10 (отлично)</t>
+          <t>6 из 9. Как помогли с техникой, доступами и рабочим местом? - от 1 (плохо) до 10 (отлично)</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>7 из 9. Вовремя ли выдали доступы? — от 1 (были задержки) до 10 (без задержек)</t>
+          <t>7 из 9. Вовремя ли выдали доступы? - от 1 (были задержки) до 10 (без задержек)</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr"/>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>8 из 9. Как HR помогает с вопросами сейчас? — от 1 (плохо) до 10 (отлично)</t>
+          <t>8 из 9. Как HR помогает с вопросами сейчас? - от 1 (плохо) до 10 (отлично)</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>9 из 9. Как HR помогал с подготовкой к выходу на работу? — от 1 (плохо) до 10 (отлично)</t>
+          <t>9 из 9. Как HR помогал с подготовкой к выходу на работу? - от 1 (плохо) до 10 (отлично)</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr"/>
@@ -3078,12 +3078,12 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Привет, {имя}! Сегодня ровно месяц, как ты с нами. Поздравляю — первый, самый сложный месяц позади.</t>
+          <t>Привет, {имя}! Сегодня ровно месяц, как ты с нами. Поздравляю: первый, самый сложный месяц позади.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Здравствуйте, {имя}! Сегодня ровно месяц, как вы с нами. Поздравляю — первый, самый сложный месяц позади.</t>
+          <t>Здравствуйте, {имя}! Сегодня ровно месяц, как вы с нами. Поздравляю: первый, самый сложный месяц позади.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>Убрали «Мы придаём большое значение успешной адаптации». Кнопки короче. Для «Немного отстаю» — отдельный, более спокойный ответ. /HR → /hr. Команды /hr в боте пока нет.</t>
+          <t>Убрали «Мы придаём большое значение успешной адаптации». Кнопки короче. Для «Немного отстаю»: отдельный, более спокойный ответ. /HR → /hr. Команды /hr в боте пока нет.</t>
         </is>
       </c>
     </row>
@@ -3189,12 +3189,12 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Ничего страшного, так бывает. Если нужна помощь — пиши.</t>
+          <t>Ничего страшного, так бывает. Если нужна помощь, пиши.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Ничего страшного, так бывает. Если нужна помощь — пишите.</t>
+          <t>Ничего страшного, так бывает. Если нужна помощь, пишите.</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -3222,12 +3222,12 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Спасибо, что честно говоришь. Напиши, что мешает, — передам в отдел подбора.</t>
+          <t>Спасибо, что честно говоришь. Напиши, что мешает, передам в отдел подбора.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Спасибо, что честно говорите. Напишите, что мешает, — передам в отдел подбора.</t>
+          <t>Спасибо, что честно говорите. Напишите, что мешает, передам в отдел подбора.</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -3259,12 +3259,12 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Привет, {имя}! Напоминаю: через 2–3 дня у тебя встреча с менеджером по подбору — обсудите, как идёт адаптационный план. Детали пришлёт твой куратор из отдела по подбору и адаптации персонала 🙂</t>
+          <t>Привет, {имя}! Напоминаю: через 2–3 дня у тебя встреча с менеджером по подбору: обсудите, как идёт адаптационный план. Детали пришлёт твой куратор из отдела по подбору и адаптации персонала 🙂</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Здравствуйте, {имя}! Напоминаю: через 2–3 дня у вас встреча с менеджером по подбору — обсудите, как идёт адаптационный план. Детали пришлёт ваш куратор из отдела по подбору и адаптации персонала 🙂</t>
+          <t>Здравствуйте, {имя}! Напоминаю: через 2–3 дня у вас встреча с менеджером по подбору: обсудите, как идёт адаптационный план. Детали пришлёт ваш куратор из отдела по подбору и адаптации персонала 🙂</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Было «закреплённый за тобой Сотрудник Отдела по подбору и адаптации персонала» — канцелярит и лишние заглавные. Время в исходнике не указано, взяли 10:00.</t>
+          <t>Было «закреплённый за тобой Сотрудник Отдела по подбору и адаптации персонала»: канцелярит и лишние заглавные. Время в исходнике не указано, взяли 10:00.</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Я собрал подборку фильмов на выходные — все про первые шаги на новой работе.
+          <t>Я собрал подборку фильмов на выходные: все про первые шаги на новой работе.
 🎬 «Дьявол носит Prada» (2006). Выпускница журфака становится ассистенткой самой требовательной начальницы в мире моды и по ходу понимает, чего хочет сама.
 🎬 «Стажёр» (2015). 70-летний Бен идёт стажёром в онлайн-магазин одежды и доказывает, что учиться новому можно в любом возрасте. Тёплое, доброе кино.
 🎬 «В погоне за счастьем» (2006). Отец-одиночка в трудном положении проходит неоплачиваемую стажировку в брокерской компании, чтобы получить работу мечты.
@@ -3347,7 +3347,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Я собрал для вас подборку фильмов на выходные — все про первые шаги на новой работе.
+          <t>Я собрал для вас подборку фильмов на выходные: все про первые шаги на новой работе.
 🎬 «Дьявол носит Prada» (2006). Выпускница журфака становится ассистенткой самой требовательной начальницы в мире моды и по ходу понимает, чего хочет сама.
 🎬 «Стажёр» (2015). 70-летний Бен идёт стажёром в онлайн-магазин одежды и доказывает, что учиться новому можно в любом возрасте. Тёплое, доброе кино.
 🎬 «В погоне за счастьем» (2006). Отец-одиночка в трудном положении проходит неоплачиваемую стажировку в брокерской компании, чтобы получить работу мечты.
@@ -3360,7 +3360,7 @@
       <c r="J75" s="2" t="inlineStr"/>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>Сократили описания. Убрали «Мне бы в небо»: главный герой этого фильма увольняет людей — странная рекомендация новичку. Если нужен пятый фильм, пусть его выберет HR. Героиня последнего фильма работает в финансовой компании, а не в консалтинговой — поправили.</t>
+          <t>Сократили описания. Убрали «Мне бы в небо»: главный герой этого фильма увольняет людей - странная рекомендация новичку. Если нужен пятый фильм, пусть его выберет HR. Героиня последнего фильма работает в финансовой компании, а не в консалтинговой, поправили.</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>Пометка про вложение — в скобках.</t>
+          <t>Пометка про вложение - в скобках.</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       <c r="J77" s="2" t="inlineStr"/>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>Было «чтобы ты смог поделиться» — мужской род. Сказали, сколько вопросов.</t>
+          <t>Было «чтобы ты смог поделиться»: мужской род. Сказали, сколько вопросов.</t>
         </is>
       </c>
     </row>
@@ -3511,12 +3511,12 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Жаль, что работа пока не радует. Если мы с коллегами можем что-то изменить, расскажи — вместе подумаем, как сделать работу комфортнее.</t>
+          <t>Жаль, что работа пока не радует. Если мы с коллегами можем что-то изменить, расскажи, вместе подумаем, как сделать работу комфортнее.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Жаль, что работа пока не радует. Если мы с коллегами можем что-то изменить, расскажите — вместе подумаем, как сделать работу комфортнее.</t>
+          <t>Жаль, что работа пока не радует. Если мы с коллегами можем что-то изменить, расскажите, вместе подумаем, как сделать работу комфортнее.</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -3552,12 +3552,12 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Так бывает: много задач, сжатые сроки, высокие ожидания. Но постоянное напряжение — не норма, и терпеть его не нужно. Расскажи, что происходит, — передам в отдел подбора, вместе придумаем, как разгрузить.</t>
+          <t>Так бывает: много задач, сжатые сроки, высокие ожидания. Но постоянное напряжение - не норма, и терпеть его не нужно. Расскажи, что происходит, передам в отдел подбора, вместе придумаем, как разгрузить.</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Так бывает: много задач, сжатые сроки, высокие ожидания. Но постоянное напряжение — не норма, и терпеть его не нужно. Расскажите, что происходит, — передам в отдел подбора, вместе придумаем, как разгрузить.</t>
+          <t>Так бывает: много задач, сжатые сроки, высокие ожидания. Но постоянное напряжение - не норма, и терпеть его не нужно. Расскажите, что происходит, передам в отдел подбора, вместе придумаем, как разгрузить.</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -3634,7 +3634,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Поддержка на старте очень важна. Я всегда на связи, но некоторые вопросы мне не решить — тут поможет рекрутер.</t>
+          <t>Поддержка на старте очень важна. Я всегда на связи, но некоторые вопросы мне не решить: тут поможет рекрутер.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr"/>
@@ -3798,12 +3798,12 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Жаль, что работа пока не радует. Если мы с коллегами можем что-то изменить, расскажи — вместе подумаем, как сделать работу комфортнее.</t>
+          <t>Жаль, что работа пока не радует. Если мы с коллегами можем что-то изменить, расскажи, вместе подумаем, как сделать работу комфортнее.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Жаль, что работа пока не радует. Если мы с коллегами можем что-то изменить, расскажите — вместе подумаем, как сделать работу комфортнее.</t>
+          <t>Жаль, что работа пока не радует. Если мы с коллегами можем что-то изменить, расскажите, вместе подумаем, как сделать работу комфортнее.</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -3839,12 +3839,12 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Так бывает: много задач, сжатые сроки, высокие ожидания. Но постоянное напряжение — не норма, и терпеть его не нужно. Расскажи, что происходит, — передам в отдел подбора, вместе придумаем, как разгрузить.</t>
+          <t>Так бывает: много задач, сжатые сроки, высокие ожидания. Но постоянное напряжение - не норма, и терпеть его не нужно. Расскажи, что происходит, передам в отдел подбора, вместе придумаем, как разгрузить.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Так бывает: много задач, сжатые сроки, высокие ожидания. Но постоянное напряжение — не норма, и терпеть его не нужно. Расскажите, что происходит, — передам в отдел подбора, вместе придумаем, как разгрузить.</t>
+          <t>Так бывает: много задач, сжатые сроки, высокие ожидания. Но постоянное напряжение - не норма, и терпеть его не нужно. Расскажите, что происходит, передам в отдел подбора, вместе придумаем, как разгрузить.</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Поддержка на старте очень важна. Я всегда на связи, но некоторые вопросы мне не решить — тут поможет рекрутер.</t>
+          <t>Поддержка на старте очень важна. Я всегда на связи, но некоторые вопросы мне не решить: тут поможет рекрутер.</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr"/>
@@ -4045,7 +4045,7 @@
       <c r="J92" s="2" t="inlineStr"/>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>Сократили вдвое, смысл веток сохранили. Эти три ответа — кандидаты в «красные флаги»: в нашем решении HR получает уведомление сразу, не дожидаясь отчёта. Здесь только благодарность, ответы на варианты стоят ветками у шагов 55 и 56.</t>
+          <t>Сократили вдвое, смысл веток сохранили. Эти три ответа - кандидаты в «красные флаги»: в нашем решении HR получает уведомление сразу, не дожидаясь отчёта. Здесь только благодарность, ответы на варианты стоят ветками у шагов 55 и 56.</t>
         </is>
       </c>
     </row>
@@ -4069,12 +4069,12 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Привет, {имя}! Давно не писал — не хотел отвлекать от работы. Но такую дату пропустить не мог: начался третий месяц, ты на финишной прямой испытательного срока.</t>
+          <t>Привет, {имя}! Давно не писал, не хотел отвлекать от работы. Но такую дату пропустить не мог: начался третий месяц, ты на финишной прямой испытательного срока.</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Здравствуйте, {имя}! Давно не писал — не хотел отвлекать от работы. Но такую дату пропустить не мог: начался третий месяц, вы на финишной прямой испытательного срока.</t>
+          <t>Здравствуйте, {имя}! Давно не писал, не хотел отвлекать от работы. Но такую дату пропустить не мог: начался третий месяц, вы на финишной прямой испытательного срока.</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr"/>
@@ -4110,7 +4110,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Привет, {имя}! Пока мы не виделись, я собрал ещё одну подборку — книги о работе и о себе. Вдруг что-то зацепит 😉
+          <t>Привет, {имя}! Пока мы не виделись, я собрал ещё одну подборку: книги о работе и о себе. Вдруг что-то зацепит 😉
 📘 «Найти своё призвание», Кен Робинсон. Чем работа «потому что надо» отличается от дела, к которому лежит душа. Есть упражнения, чтобы разобраться в себе.
 📘 «Кради как художник», Остин Клеон. Короткая книга на случай, когда кончились идеи.
 📘 «Между надо и хочу», Эль Луна. Книга-собеседник для тех, кто на распутье: разобрать свои «надо», понять свои «хочу» и начать действовать.
@@ -4118,12 +4118,12 @@
 📘 «Работа твоей мечты», Барбара Шер. Советы о том, как найти работу по душе. Местами наивно, но помогает посмотреть на карьеру шире.
 📘 «Работа», Байрон Кейти. Метод четырёх вопросов для работы над собой.
 📘 «Great work. Как найти вдохновение, полюбить свою работу и начать зарабатывать», Дэвид Стерт. Пять практических навыков, которые помогают делать работу, которую замечают и ценят.
-📘 «Энергия — новая валюта», Леонид Кроль. Как распределять силы и где их брать — с примерами и практическими советами.</t>
+📘 «Энергия - новая валюта», Леонид Кроль. Как распределять силы и где их брать, с примерами и практическими советами.</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Здравствуйте, {имя}! Пока мы не виделись, я собрал ещё одну подборку — книги о работе и о себе. Вдруг что-то зацепит 😉
+          <t>Здравствуйте, {имя}! Пока мы не виделись, я собрал ещё одну подборку: книги о работе и о себе. Вдруг что-то зацепит 😉
 📘 «Найти своё призвание», Кен Робинсон. Чем работа «потому что надо» отличается от дела, к которому лежит душа. Есть упражнения, чтобы разобраться в себе.
 📘 «Кради как художник», Остин Клеон. Короткая книга на случай, когда кончились идеи.
 📘 «Между надо и хочу», Эль Луна. Книга-собеседник для тех, кто на распутье: разобрать свои «надо», понять свои «хочу» и начать действовать.
@@ -4131,7 +4131,7 @@
 📘 «Работа твоей мечты», Барбара Шер. Советы о том, как найти работу по душе. Местами наивно, но помогает посмотреть на карьеру шире.
 📘 «Работа», Байрон Кейти. Метод четырёх вопросов для работы над собой.
 📘 «Great work. Как найти вдохновение, полюбить свою работу и начать зарабатывать», Дэвид Стерт. Пять практических навыков, которые помогают делать работу, которую замечают и ценят.
-📘 «Энергия — новая валюта», Леонид Кроль. Как распределять силы и где их брать — с примерами и практическими советами.</t>
+📘 «Энергия - новая валюта», Леонид Кроль. Как распределять силы и где их брать, с примерами и практическими советами.</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr"/>
@@ -4139,7 +4139,7 @@
       <c r="J94" s="2" t="inlineStr"/>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>Описания сократили. Убрали книгу «Ты способна на большее. 12 привычек, которые мешают женщинам сделать карьеру»: бот пишет всем новичкам, а книга адресована только женщинам. Названия остальных книг оставили как в исходнике — перед запуском сверить с изданиями. В исходнике «для офисных сотрудников», тега не было.</t>
+          <t>Описания сократили. Убрали книгу «Ты способна на большее. 12 привычек, которые мешают женщинам сделать карьеру»: бот пишет всем новичкам, а книга адресована только женщинам. Названия остальных книг оставили как в исходнике: перед запуском сверить с изданиями. В исходнике «для офисных сотрудников», тега не было.</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>Служебная пометка — в скобках. Текст наш: в исходнике была только открытка.</t>
+          <t>Служебная пометка - в скобках. Текст наш: в исходнике была только открытка.</t>
         </is>
       </c>
     </row>
@@ -4204,12 +4204,12 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>{имя}, привет! Три месяца пролетели — испытательный срок подошёл к концу. Пока впечатления свежие, поделишься ими? Это займёт несколько минут.</t>
+          <t>{имя}, привет! Три месяца пролетели: испытательный срок подошёл к концу. Пока впечатления свежие, поделишься ими? Это займёт несколько минут.</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>{имя}, здравствуйте! Три месяца пролетели — испытательный срок подошёл к концу. Пока впечатления свежие, поделитесь ими? Это займёт несколько минут.</t>
+          <t>{имя}, здравствуйте! Три месяца пролетели: испытательный срок подошёл к концу. Пока впечатления свежие, поделитесь ими? Это займёт несколько минут.</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr"/>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>Было «Дорогой Х» — мужской род. Убрали «Ты только начинаешь познавать нашу компанию».</t>
+          <t>Было «Дорогой Х»: мужской род. Убрали «Ты только начинаешь познавать нашу компанию».</t>
         </is>
       </c>
     </row>
@@ -4393,12 +4393,12 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Можно спросить, что вызывает сомнения? Напиши здесь — или расскажи рекрутеру лично, если так удобнее.</t>
+          <t>Можно спросить, что вызывает сомнения? Напиши здесь, или расскажи рекрутеру лично, если так удобнее.</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Можно спросить, что вызывает сомнения? Напишите здесь — или расскажите рекрутеру лично, если так удобнее.</t>
+          <t>Можно спросить, что вызывает сомнения? Напишите здесь, или расскажите рекрутеру лично, если так удобнее.</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr"/>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Ещё несколько оценок — по шкале от 1 до 10.</t>
+          <t>Ещё несколько оценок - по шкале от 1 до 10.</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr"/>
@@ -4468,7 +4468,7 @@
       <c r="J103" s="2" t="inlineStr"/>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>Как в строке 47: вопросы были на «вы», сделали две версии, логику «ниже 8 — уточнить» сохранили. Добавили вводную фразу, чтобы список не начинался без предупреждения. Девять оценок разбиты на шаги 64.1-64.9.</t>
+          <t>Как в строке 47: вопросы были на «вы», сделали две версии, логику «ниже 8 - уточнить» сохранили. Добавили вводную фразу, чтобы список не начинался без предупреждения. Девять оценок разбиты на шаги 64.1-64.9.</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4492,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>1 из 9. Насколько комфортна нагрузка? — от 1 (очень некомфортно) до 10 (полностью комфортно)</t>
+          <t>1 из 9. Насколько комфортна нагрузка? - от 1 (очень некомфортно) до 10 (полностью комфортно)</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr"/>
@@ -4525,7 +4525,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2 из 9. Совпали ли ожидания от работы с реальностью? — от 1 (разочаровали) до 10 (превзошли ожидания)</t>
+          <t>2 из 9. Совпали ли ожидания от работы с реальностью? - от 1 (разочаровали) до 10 (превзошли ожидания)</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr"/>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>3 из 9. Хватает ли информации, чтобы хорошо делать свою работу? — Да / Нет</t>
+          <t>3 из 9. Хватает ли информации, чтобы хорошо делать свою работу? - Да / Нет</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr"/>
@@ -4595,7 +4595,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>4 из 9. Насколько руководитель доступен для вопросов и обратной связи? — от 1 (недоступен) до 10 (всегда на связи)</t>
+          <t>4 из 9. Насколько руководитель доступен для вопросов и обратной связи? - от 1 (недоступен) до 10 (всегда на связи)</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr"/>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>5 из 9. Насколько полезна обратная связь от руководителя? — от 1 (её нет) до 10 (подробная и по делу)</t>
+          <t>5 из 9. Насколько полезна обратная связь от руководителя? - от 1 (её нет) до 10 (подробная и по делу)</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
@@ -4661,7 +4661,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>6 из 9. Помогают ли коллеги, когда возникают вопросы или сложности? — от 1 (не помогают) до 10 (всегда помогают)</t>
+          <t>6 из 9. Помогают ли коллеги, когда возникают вопросы или сложности? - от 1 (не помогают) до 10 (всегда помогают)</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr"/>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>7 из 9. Как складывается работа с другими подразделениями? — от 1 (плохо) до 10 (отлично)</t>
+          <t>7 из 9. Как складывается работа с другими подразделениями? - от 1 (плохо) до 10 (отлично)</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr"/>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>8 из 9. Как HR помогает с вопросами? — от 1 (плохо) до 10 (отлично)</t>
+          <t>8 из 9. Как HR помогает с вопросами? - от 1 (плохо) до 10 (отлично)</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr"/>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>9 из 9. Удалось ли выполнить задачи испытательного срока? — от 1 (совсем не удалось) до 10 (полностью)</t>
+          <t>9 из 9. Удалось ли выполнить задачи испытательного срока? - от 1 (совсем не удалось) до 10 (полностью)</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
@@ -4806,7 +4806,7 @@
       <c r="J113" s="2" t="inlineStr"/>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>Было «Что порекомендуешь улучшить для более комфортной адаптации сотрудника?» — тяжело читается.</t>
+          <t>Было «Что порекомендуешь улучшить для более комфортной адаптации сотрудника?»: тяжело читается.</t>
         </is>
       </c>
     </row>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>И напоследок — плейлист для концентрации 🎶</t>
+          <t>И напоследок: плейлист для концентрации 🎶</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr"/>
@@ -4880,7 +4880,7 @@
       <c r="J115" s="2" t="inlineStr"/>
       <c r="K115" s="2" t="inlineStr">
         <is>
-          <t>Убрали из ссылки «?lang=en» — у русскоязычного пользователя страница должна открываться на русском. Ссылка стала кнопкой: в МАКС нельзя сделать ссылкой одно слово.</t>
+          <t>Убрали из ссылки «?lang=en»: у русскоязычного пользователя страница должна открываться на русском. Ссылка стала кнопкой: в МАКС нельзя сделать ссылкой одно слово.</t>
         </is>
       </c>
     </row>
@@ -4904,14 +4904,14 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Кажется, всё: вопросы заданы, материалы отправлены. Пора прощаться — по крайней мере, на время.
+          <t>Кажется, всё: вопросы заданы, материалы отправлены. Пора прощаться, по крайней мере, на время.
 Надеюсь, с моей помощью первые месяцы прошли чуть легче. Если понадобится помощь, ты знаешь, где найти коллег из HR. А я рад, что был рядом.
 До встречи, {имя}! 👋</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>Кажется, всё: вопросы заданы, материалы отправлены. Пора прощаться — по крайней мере, на время.
+          <t>Кажется, всё: вопросы заданы, материалы отправлены. Пора прощаться, по крайней мере, на время.
 Надеюсь, с моей помощью первые месяцы прошли чуть легче. Если понадобится помощь, вы знаете, где найти коллег из HR. А я рад, что был рядом.
 До встречи, {имя}! 👋</t>
         </is>
@@ -4953,12 +4953,12 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>Хороший вопрос, но точного ответа в документах компании я не нашёл. Гадать не хочу — передам вопрос коллегам из отдела подбора, они ответят прямо здесь.</t>
+          <t>Хороший вопрос, но точного ответа в документах компании я не нашёл. Гадать не хочу, передам вопрос коллегам из отдела подбора, они ответят прямо здесь.</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>Хороший вопрос, но точного ответа в документах компании я не нашёл. Гадать не хочу — передам вопрос коллегам из отдела подбора, они ответят вам прямо здесь.</t>
+          <t>Хороший вопрос, но точного ответа в документах компании я не нашёл. Гадать не хочу, передам вопрос коллегам из отдела подбора, они ответят вам прямо здесь.</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr"/>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="K117" s="2" t="inlineStr">
         <is>
-          <t>Раньше бот так отвечал на любой вопрос. В новом решении это запасной ответ: сначала ИИ ищет ответ в базе знаний и отвечает со ссылкой на документ, и только если не нашёл — эта реплика. Не шаг по времени: так бот отвечает, когда передал вопрос HR.</t>
+          <t>Раньше бот так отвечал на любой вопрос. В новом решении это запасной ответ: сначала ИИ ищет ответ в базе знаний и отвечает со ссылкой на документ, и только если не нашёл - эта реплика. Не шаг по времени: так бот отвечает, когда передал вопрос HR.</t>
         </is>
       </c>
     </row>
@@ -5011,7 +5011,7 @@
       </c>
       <c r="K118" s="2" t="inlineStr">
         <is>
-          <t>Было «ты не прошел опрос» — звучит как упрёк и в мужском роде. Добавили кнопку, чтобы продолжить с того же места. Не шаг по времени: текст напоминания про вопрос без ответа. Кнопки «Продолжить опрос» нет.</t>
+          <t>Было «ты не прошел опрос»: звучит как упрёк и в мужском роде. Добавили кнопку, чтобы продолжить с того же места. Не шаг по времени: текст напоминания про вопрос без ответа. Кнопки «Продолжить опрос» нет.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
workplaces with hours, recruiter schedule and reminders, answers in working time, late newcomers get required steps, dashboard
</commit_message>
<xml_diff>
--- a/scenario/scenario.xlsx
+++ b/scenario/scenario.xlsx
@@ -56,7 +56,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -70,6 +70,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:N118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -448,7 +449,10 @@
     <col width="32" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="55" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,7 +506,22 @@
           <t>Картинка</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Обязательный</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Кратко на «ты»</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Кратко на «вы»</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
@@ -540,7 +559,12 @@
           <t>img_02.png</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Это сообщение уходит до вопроса «на ты или на вы», поэтому оно на «вы» в обеих версиях. Убрали «Привет-привет-привет», пять эмодзи и общие слова про «путешествие навстречу успехам». Оставили, чем бот реально поможет.</t>
         </is>
@@ -577,7 +601,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>Короче и без двойного вопроса. Строки 5 и 6 исходника: вопрос и кнопки в одном шаге.</t>
         </is>
@@ -614,7 +643,12 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>«Х» заменили на переменную {имя}. Ответ зависит от выбора. Стоит после шага 5 и ждёт выбора, поэтому уходит уже в нужном регистре.</t>
         </is>
@@ -657,7 +691,7 @@
           <t>img_01.png</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Было два варианта на выбор, объединили в один. Добавили главное: боту можно задавать вопросы в любой момент.</t>
         </is>
@@ -720,7 +754,12 @@
           <t>img_03.png</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Было «чтобы ты пришел подготовленный»: мужской род и канцелярит. Добавили, что делать, если документа нет. Список в колонке J: без «Вашего», с единым оформлением. Список документов из колонки J добавлен в конец текста.</t>
         </is>
@@ -785,7 +824,12 @@
           <t>img_03.png</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>Как в строке 9. Для GTP в списке есть фото 3×4, для GrPP и Luzhniki - нет. Уточнить у HR, так и задумано или фото нужно всем. Список документов из колонки J добавлен в конец текста.</t>
         </is>
@@ -822,7 +866,7 @@
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>Короче. Текст без «ты/вы», подходит обеим версиям. Что прислать после «да», в исходнике нет, поэтому шаг без кнопок: ответ новичка разберёт ИИ по базе знаний или передаст рекрутеру. Когда HR даст материалы, сделать кнопки и ветку.</t>
         </is>
@@ -859,7 +903,7 @@
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>Как в строке 11. Что прислать после «да», в исходнике нет, поэтому шаг без кнопок: ответ новичка разберёт ИИ по базе знаний или передаст рекрутеру. Когда HR даст материалы, сделать кнопки и ветку.</t>
         </is>
@@ -896,7 +940,7 @@
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Короче, без «ты легко спланировал» (мужской род). Что прислать после «да», в исходнике нет, поэтому шаг без кнопок: ответ новичка разберёт ИИ по базе знаний или передаст рекрутеру. Когда HR даст материалы, сделать кнопки и ветку.</t>
         </is>
@@ -941,7 +985,7 @@
       <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>Было от лица бота («я горжусь, что работаю в компании», «даже я хожу на тренинги») и с фактами, которых нет в материалах: «миллионы людей», «филиалы по всей России и СНГ». Оставили только то, что есть в материалах кейса: 35 лет, около 8500 человек, чем занимается компания. Пункт в скобках заполняет HR.</t>
         </is>
@@ -980,7 +1024,7 @@
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Чуть короче, «Х» → {имя}.</t>
         </is>
@@ -1021,7 +1065,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>Кнопка «Готов/Готова» → «Всё готово», без рода. Убрали шутку «я сам через это проходил, когда меня создавали»: она обесценивает волнение. Добавили, что боту можно писать. Время в исходнике не указано, взяли 10:00. Ответ сохраняется как опрос.</t>
         </is>
@@ -1054,7 +1098,7 @@
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1083,7 +1127,7 @@
       <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1112,7 +1156,7 @@
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1141,7 +1185,7 @@
       <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>Строка 16, «дальше всем»: уходит после ответа на шаг 16.</t>
         </is>
@@ -1202,7 +1246,7 @@
           <t>img_03.png</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>Короче. Текст из колонки D («Напомнить кандидату о списке документов…») перенесли в колонку C: это информационный повод, а не тег сотрудника. Тег пустой - значит, для всех площадок. Список документов из колонки J добавлен в конец текста.</t>
         </is>
@@ -1245,7 +1289,7 @@
           <t>img_04.png</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>Сократили. Убрали общие фразы («вносить свой вклад в наше общее дело», «создать комфортные условия»), оставили главное: спрашивать можно и нужно.</t>
         </is>
@@ -1282,7 +1326,7 @@
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>Короче, без «ты/вы». Что прислать после «да», в исходнике нет, поэтому шаг без кнопок: ответ новичка разберёт ИИ по базе знаний или передаст рекрутеру. Когда HR даст материалы, сделать кнопки и ветку.</t>
         </is>
@@ -1319,7 +1363,7 @@
       <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>Как в строке 20. Что прислать после «да», в исходнике нет, поэтому шаг без кнопок: ответ новичка разберёт ИИ по базе знаний или передаст рекрутеру. Когда HR даст материалы, сделать кнопки и ветку.</t>
         </is>
@@ -1364,7 +1408,22 @@
       </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Всё ли готово на рабочем месте: техника, учётная запись, доступы?</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>Всё ли готово на рабочем месте: техника, учётная запись, доступы?</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>Убрали «Тебе предстоит многое узнать» и «Ничего страшного!». Кнопка «Нет» → «Чего-то не хватает». Добавили, что бот передаст проблему рекрутеру, а не только отправит к руководителю.</t>
         </is>
@@ -1405,7 +1464,7 @@
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1442,7 +1501,7 @@
       <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1483,7 +1542,22 @@
       </c>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Всё ли готово на рабочем месте: оборудование и доступы?</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>Всё ли готово на рабочем месте: оборудование и доступы?</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>В исходнике в одном сообщении были и «ты», и «вашему», «у вас». Теперь каждая версия в своём регистре.</t>
         </is>
@@ -1524,7 +1598,7 @@
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1561,7 +1635,7 @@
       <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1598,7 +1672,7 @@
           <t>card_1.png</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>Было «Дарю небольшую открытку!». Служебные пометки для бота - в квадратных скобках.</t>
         </is>
@@ -1635,7 +1709,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>Команда /Food → /food (строчными, как принято для команд). Добавили, что можно спросить своими словами: это понимает ИИ-модуль. Кнопка «Да, подскажи» стала «Да!»: колонка кнопок общая для «ты» и «вы». Команды /food в боте пока нет, работает вопрос своими словами.</t>
         </is>
@@ -1672,7 +1746,7 @@
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>Правка движка: убрали /food, такой команды в боте нет, про еду новичок спрашивает своими словами.</t>
         </is>
@@ -1714,7 +1788,7 @@
           <t>img_05.png</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>Без «ты/вы». Пометка про вложение - в скобках. PDF бот не отправляет, только картинки: список лучше вписать текстом.</t>
         </is>
@@ -1756,7 +1830,7 @@
           <t>img_05.png</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>Как в строке 26. PDF бот не отправляет, только картинки: список лучше вписать текстом.</t>
         </is>
@@ -1798,7 +1872,7 @@
           <t>img_05.png</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>Как в строке 26. PDF бот не отправляет, только картинки: список лучше вписать текстом.</t>
         </is>
@@ -1831,7 +1905,7 @@
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>Было «ты уже немного освоился»: мужской род. Сократили.</t>
         </is>
@@ -1877,7 +1951,18 @@
           <t>img_06.png</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Справочник контактов коллег: https://my.polyplastic.ru/employees/Pages/address-book.aspx (открывается с рабочего компьютера).</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>Прямо сказали, что с телефона справочник не откроется: бот присылает ссылку в мессенджер, и новичок будет пробовать открыть её с телефона. Ссылка продублирована кнопкой.</t>
         </is>
@@ -1919,7 +2004,18 @@
           <t>img_06.png</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Справочник контактов коллег: http://ats/ (открывается с рабочего компьютера).</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>Как в строке 30. Без кнопки: адрес http://ats/ внутренний.</t>
         </is>
@@ -1960,7 +2056,7 @@
       <c r="H37" s="2" t="inlineStr"/>
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="N37" s="2" t="inlineStr">
         <is>
           <t>Миссию оставили дословно: это официальная формулировка. Убрали «Мы ценим каждого сотрудника и верим, что только вместе…»: общие слова, которые есть в любом приветствии.</t>
         </is>
@@ -2003,7 +2099,7 @@
           <t>img_10.png</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr">
         <is>
           <t>Убрали «я уверен, что ты успешно справился»: мужской род, и бот не знает, как прошёл день. Добавили открытый вопрос: ответ разберёт ИИ-модуль настроений. В исходнике «для сотрудников офиса», тега не было: если нужно, поставить тег.</t>
         </is>
@@ -2042,7 +2138,7 @@
       <c r="H39" s="2" t="inlineStr"/>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr">
         <is>
           <t>Было «Составь, пожалуйста, краткое описание… (образец)»: звучало как задание. Объяснили зачем, фото - по желанию, добавили образец и согласование перед публикацией. Черновик знакомства собирает ИИ из ответа новичка. В исходнике «по отмашке рекрутера», сейчас уходит всем. Бот сохраняет ответ, сам знакомство не публикует.
 Правка движка: бот не принимает фото и не показывает черновик, ответ сохраняется и уходит рекрутеру.</t>
@@ -2080,7 +2176,7 @@
       <c r="H40" s="2" t="inlineStr"/>
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr">
         <is>
           <t>Короче.</t>
         </is>
@@ -2125,7 +2221,22 @@
           <t>img_07.png</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>У тебя есть адаптационный план на испытательный срок: если его ещё не показали, попроси у руководителя.</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>У вас есть адаптационный план на испытательный срок: если его ещё не показали, попросите у руководителя.</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>«Не бойся обращаться» → «это нормально». Убрали «Надеюсь, ты уже чуть лучше понимаешь наши ценности и правила». План бот сам не прикладывает, см. пометку [HR: ...].
 Правка движка: убрали «Вот он.», плана во вложении пока нет.</t>
@@ -2163,7 +2274,7 @@
       <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>Без «ты/вы», короче. Что прислать после «да», в исходнике нет, поэтому шаг без кнопок: ответ новичка разберёт ИИ по базе знаний или передаст рекрутеру. Когда HR даст материалы, сделать кнопки и ветку.</t>
         </is>
@@ -2200,7 +2311,7 @@
       <c r="H43" s="2" t="inlineStr"/>
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="N43" s="2" t="inlineStr">
         <is>
           <t>Было «предлагаем пройти тебе опрос». Сказали, сколько вопросов и сколько времени это займёт: так больше людей доходит до конца.</t>
         </is>
@@ -2237,7 +2348,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr"/>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="N44" s="2" t="inlineStr">
         <is>
           <t>Логика веток та же. «Я буду благодарен, если ты поделишься» → прямой вопрос. Добавили номер вопроса «1 из 3». Кнопок «Написать рекрутеру» пока нет: у бота нет ссылки на личный диалог с рекрутером.</t>
         </is>
@@ -2270,7 +2381,7 @@
       <c r="H45" s="2" t="inlineStr"/>
       <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="inlineStr"/>
-      <c r="K45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2303,7 +2414,7 @@
       <c r="H46" s="2" t="inlineStr"/>
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2340,7 +2451,7 @@
       </c>
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="inlineStr"/>
-      <c r="K47" s="2" t="inlineStr">
+      <c r="N47" s="2" t="inlineStr">
         <is>
           <t>Было «ты вышел на работу в период большой нагрузки»: мужской род. «Не бойся поднять этот вопрос» → «скажи об этом».</t>
         </is>
@@ -2377,7 +2488,7 @@
       <c r="H48" s="2" t="inlineStr"/>
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr"/>
-      <c r="K48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2410,7 +2521,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr"/>
-      <c r="K49" s="2" t="inlineStr">
+      <c r="N49" s="2" t="inlineStr">
         <is>
           <t>Кнопка «Пока ничего не понял» → «Пока ничего не понятно», без рода. Ответы сократили, логика веток та же.</t>
         </is>
@@ -2443,7 +2554,7 @@
       <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr"/>
-      <c r="K50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2476,7 +2587,7 @@
       <c r="H51" s="2" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="inlineStr"/>
-      <c r="K51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2509,7 +2620,7 @@
       <c r="H52" s="2" t="inlineStr"/>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr"/>
-      <c r="K52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2538,7 +2649,7 @@
       <c r="H53" s="2" t="inlineStr"/>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="inlineStr"/>
-      <c r="K53" s="2" t="inlineStr">
+      <c r="N53" s="2" t="inlineStr">
         <is>
           <t>Без изменений по смыслу.</t>
         </is>
@@ -2579,7 +2690,7 @@
       <c r="H54" s="2" t="inlineStr"/>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr"/>
-      <c r="K54" s="2" t="inlineStr">
+      <c r="N54" s="2" t="inlineStr">
         <is>
           <t>Было «Сегодня я хотел бы рассказать тебе об еще одном аспекте работы в нашей компании»: канцелярит. Время в исходнике не указано, взяли 10:00.</t>
         </is>
@@ -2620,7 +2731,7 @@
           <t>img_11.png</t>
         </is>
       </c>
-      <c r="K55" s="2" t="inlineStr">
+      <c r="N55" s="2" t="inlineStr">
         <is>
           <t>Убрали «важная часть культуры компании» и «дружелюбную и поддерживающую атмосферу». Оставили конкретику: какие бывают праздники.</t>
         </is>
@@ -2661,7 +2772,7 @@
           <t>photo_1.png</t>
         </is>
       </c>
-      <c r="K56" s="2" t="inlineStr">
+      <c r="N56" s="2" t="inlineStr">
         <is>
           <t>Пометка про вложение - в скобках. В исходнике картинка «ФОТО», назвали photo_1.png.</t>
         </is>
@@ -2702,7 +2813,7 @@
       <c r="H57" s="2" t="inlineStr"/>
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="inlineStr"/>
-      <c r="K57" s="2" t="inlineStr">
+      <c r="N57" s="2" t="inlineStr">
         <is>
           <t>Короче.</t>
         </is>
@@ -2743,7 +2854,7 @@
           <t>img_14.png</t>
         </is>
       </c>
-      <c r="K58" s="2" t="inlineStr">
+      <c r="N58" s="2" t="inlineStr">
         <is>
           <t>Вопросы были на «вы» в боте на «ты»: теперь две версии. Шкалы и правило «ниже 8 - уточнить причину» сохранили. В МАКС нет встроенных опросов: шкала 1–10 - это два ряда по 5 кнопок. Предлагаем сократить до 3 главных вопросов с уточнением только там, где оценка низкая (см. описание решения). Девять вопросов разбиты на шаги 47.1-47.9: «да/нет» это опрос, оценки это шкала. При «Нет» или оценке ниже 8 бот спрашивает, что не так.</t>
         </is>
@@ -2788,7 +2899,7 @@
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
-      <c r="K59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2825,7 +2936,7 @@
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2858,7 +2969,7 @@
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2891,7 +3002,7 @@
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
-      <c r="K62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2924,7 +3035,7 @@
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
-      <c r="K63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2957,7 +3068,7 @@
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
-      <c r="K64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2990,7 +3101,7 @@
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
-      <c r="K65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3023,7 +3134,7 @@
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr"/>
-      <c r="K66" s="2" t="inlineStr"/>
+      <c r="N66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3056,7 +3167,7 @@
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr"/>
-      <c r="K67" s="2" t="inlineStr"/>
+      <c r="N67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3093,7 +3204,7 @@
           <t>img_10.png</t>
         </is>
       </c>
-      <c r="K68" s="2" t="inlineStr">
+      <c r="N68" s="2" t="inlineStr">
         <is>
           <t>Убрали «Так держать!» и «Пусть каждый новый месяц приносит ещё больше возможностей для развития».</t>
         </is>
@@ -3134,7 +3245,7 @@
           <t>img_07.png</t>
         </is>
       </c>
-      <c r="K69" s="2" t="inlineStr">
+      <c r="N69" s="2" t="inlineStr">
         <is>
           <t>Убрали «Мы придаём большое значение успешной адаптации». Кнопки короче. Для «Немного отстаю»: отдельный, более спокойный ответ. /HR → /hr. Команды /hr в боте пока нет.</t>
         </is>
@@ -3167,7 +3278,7 @@
       <c r="H70" s="2" t="inlineStr"/>
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="inlineStr"/>
-      <c r="K70" s="2" t="inlineStr"/>
+      <c r="N70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3200,7 +3311,7 @@
       <c r="H71" s="2" t="inlineStr"/>
       <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="inlineStr"/>
-      <c r="K71" s="2" t="inlineStr"/>
+      <c r="N71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3233,7 +3344,7 @@
       <c r="H72" s="2" t="inlineStr"/>
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr"/>
-      <c r="K72" s="2" t="inlineStr">
+      <c r="N72" s="2" t="inlineStr">
         <is>
           <t>Правка движка: убрали команду /hr, её в боте нет. Ответ новичка бот передаёт сам.</t>
         </is>
@@ -3274,7 +3385,7 @@
           <t>img_15.png</t>
         </is>
       </c>
-      <c r="K73" s="2" t="inlineStr">
+      <c r="N73" s="2" t="inlineStr">
         <is>
           <t>Было «закреплённый за тобой Сотрудник Отдела по подбору и адаптации персонала»: канцелярит и лишние заглавные. Время в исходнике не указано, взяли 10:00.</t>
         </is>
@@ -3311,7 +3422,7 @@
       <c r="H74" s="2" t="inlineStr"/>
       <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr"/>
-      <c r="K74" s="2" t="inlineStr">
+      <c r="N74" s="2" t="inlineStr">
         <is>
           <t>Отдельное приветствие перед подборкой фильмов. Можно склеить со следующим сообщением. Развели с шагом 50 по времени, чтобы не было двух «Привет» подряд.</t>
         </is>
@@ -3358,7 +3469,7 @@
       <c r="H75" s="2" t="inlineStr"/>
       <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="inlineStr"/>
-      <c r="K75" s="2" t="inlineStr">
+      <c r="N75" s="2" t="inlineStr">
         <is>
           <t>Сократили описания. Убрали «Мне бы в небо»: главный герой этого фильма увольняет людей - странная рекомендация новичку. Если нужен пятый фильм, пусть его выберет HR. Героиня последнего фильма работает в финансовой компании, а не в консалтинговой, поправили.</t>
         </is>
@@ -3399,7 +3510,7 @@
           <t>img_08.png</t>
         </is>
       </c>
-      <c r="K76" s="2" t="inlineStr">
+      <c r="N76" s="2" t="inlineStr">
         <is>
           <t>Пометка про вложение - в скобках.</t>
         </is>
@@ -3436,7 +3547,7 @@
       <c r="H77" s="2" t="inlineStr"/>
       <c r="I77" s="2" t="inlineStr"/>
       <c r="J77" s="2" t="inlineStr"/>
-      <c r="K77" s="2" t="inlineStr">
+      <c r="N77" s="2" t="inlineStr">
         <is>
           <t>Было «чтобы ты смог поделиться»: мужской род. Сказали, сколько вопросов.</t>
         </is>
@@ -3481,7 +3592,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr"/>
       <c r="J78" s="2" t="inlineStr"/>
-      <c r="K78" s="2" t="inlineStr">
+      <c r="N78" s="2" t="inlineStr">
         <is>
           <t>Варианты «поработал и ушёл», «уже устал, а задачи все валятся» переписали без рода. В МАКС нет опросов с выбором нескольких ответов: во втором вопросе кнопки работают как галочки, плюс кнопка «Готово». Три вопроса разбиты на шаги, ответы из строки 57 стали ветками. Выбрать несколько вариантов в МАКС нельзя: во втором вопросе один вариант.</t>
         </is>
@@ -3522,7 +3633,7 @@
       <c r="H79" s="2" t="inlineStr"/>
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="inlineStr"/>
-      <c r="K79" s="2" t="inlineStr">
+      <c r="N79" s="2" t="inlineStr">
         <is>
           <t>Текст из строки 57 исходника: ответ стоит сразу после кнопки, а не после всего опроса.</t>
         </is>
@@ -3563,7 +3674,7 @@
       <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="inlineStr"/>
-      <c r="K80" s="2" t="inlineStr">
+      <c r="N80" s="2" t="inlineStr">
         <is>
           <t>Текст из строки 57 исходника: ответ стоит сразу после кнопки, а не после всего опроса.</t>
         </is>
@@ -3608,7 +3719,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr"/>
       <c r="J81" s="2" t="inlineStr"/>
-      <c r="K81" s="2" t="inlineStr"/>
+      <c r="N81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3641,7 +3752,7 @@
       <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="inlineStr"/>
-      <c r="K82" s="2" t="inlineStr">
+      <c r="N82" s="2" t="inlineStr">
         <is>
           <t>Текст из строки 57 исходника: ответ стоит сразу после кнопки, а не после всего опроса.</t>
         </is>
@@ -3686,7 +3797,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr"/>
       <c r="J83" s="2" t="inlineStr"/>
-      <c r="K83" s="2" t="inlineStr"/>
+      <c r="N83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3723,7 +3834,7 @@
       <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="2" t="inlineStr"/>
       <c r="J84" s="2" t="inlineStr"/>
-      <c r="K84" s="2" t="inlineStr">
+      <c r="N84" s="2" t="inlineStr">
         <is>
           <t>Текст наш: в korsik_texts его нет.</t>
         </is>
@@ -3768,7 +3879,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr"/>
       <c r="J85" s="2" t="inlineStr"/>
-      <c r="K85" s="2" t="inlineStr">
+      <c r="N85" s="2" t="inlineStr">
         <is>
           <t>Как в строке 55, без варианта «Удалённый формат работы» (для GTP его и не было). Как шаг 55, без варианта про удалённый формат.</t>
         </is>
@@ -3809,7 +3920,7 @@
       <c r="H86" s="2" t="inlineStr"/>
       <c r="I86" s="2" t="inlineStr"/>
       <c r="J86" s="2" t="inlineStr"/>
-      <c r="K86" s="2" t="inlineStr">
+      <c r="N86" s="2" t="inlineStr">
         <is>
           <t>Текст из строки 57 исходника: ответ стоит сразу после кнопки, а не после всего опроса.</t>
         </is>
@@ -3850,7 +3961,7 @@
       <c r="H87" s="2" t="inlineStr"/>
       <c r="I87" s="2" t="inlineStr"/>
       <c r="J87" s="2" t="inlineStr"/>
-      <c r="K87" s="2" t="inlineStr">
+      <c r="N87" s="2" t="inlineStr">
         <is>
           <t>Текст из строки 57 исходника: ответ стоит сразу после кнопки, а не после всего опроса.</t>
         </is>
@@ -3895,7 +4006,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr"/>
       <c r="J88" s="2" t="inlineStr"/>
-      <c r="K88" s="2" t="inlineStr"/>
+      <c r="N88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3928,7 +4039,7 @@
       <c r="H89" s="2" t="inlineStr"/>
       <c r="I89" s="2" t="inlineStr"/>
       <c r="J89" s="2" t="inlineStr"/>
-      <c r="K89" s="2" t="inlineStr">
+      <c r="N89" s="2" t="inlineStr">
         <is>
           <t>Текст из строки 57 исходника: ответ стоит сразу после кнопки, а не после всего опроса.</t>
         </is>
@@ -3973,7 +4084,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr"/>
       <c r="J90" s="2" t="inlineStr"/>
-      <c r="K90" s="2" t="inlineStr"/>
+      <c r="N90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4010,7 +4121,7 @@
       <c r="H91" s="2" t="inlineStr"/>
       <c r="I91" s="2" t="inlineStr"/>
       <c r="J91" s="2" t="inlineStr"/>
-      <c r="K91" s="2" t="inlineStr">
+      <c r="N91" s="2" t="inlineStr">
         <is>
           <t>Текст наш: в korsik_texts его нет.</t>
         </is>
@@ -4043,7 +4154,7 @@
       <c r="H92" s="2" t="inlineStr"/>
       <c r="I92" s="2" t="inlineStr"/>
       <c r="J92" s="2" t="inlineStr"/>
-      <c r="K92" s="2" t="inlineStr">
+      <c r="N92" s="2" t="inlineStr">
         <is>
           <t>Сократили вдвое, смысл веток сохранили. Эти три ответа - кандидаты в «красные флаги»: в нашем решении HR получает уведомление сразу, не дожидаясь отчёта. Здесь только благодарность, ответы на варианты стоят ветками у шагов 55 и 56.</t>
         </is>
@@ -4084,7 +4195,7 @@
           <t>img_09.png</t>
         </is>
       </c>
-      <c r="K93" s="2" t="inlineStr">
+      <c r="N93" s="2" t="inlineStr">
         <is>
           <t>Почти без изменений, чуть короче.</t>
         </is>
@@ -4137,7 +4248,7 @@
       <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr"/>
       <c r="J94" s="2" t="inlineStr"/>
-      <c r="K94" s="2" t="inlineStr">
+      <c r="N94" s="2" t="inlineStr">
         <is>
           <t>Описания сократили. Убрали книгу «Ты способна на большее. 12 привычек, которые мешают женщинам сделать карьеру»: бот пишет всем новичкам, а книга адресована только женщинам. Названия остальных книг оставили как в исходнике: перед запуском сверить с изданиями. В исходнике «для офисных сотрудников», тега не было.</t>
         </is>
@@ -4178,7 +4289,7 @@
           <t>card_2.png</t>
         </is>
       </c>
-      <c r="K95" s="2" t="inlineStr">
+      <c r="N95" s="2" t="inlineStr">
         <is>
           <t>Служебная пометка - в скобках. Текст наш: в исходнике была только открытка.</t>
         </is>
@@ -4219,7 +4330,7 @@
           <t>img_10.png</t>
         </is>
       </c>
-      <c r="K96" s="2" t="inlineStr">
+      <c r="N96" s="2" t="inlineStr">
         <is>
           <t>Было «Дорогой Х»: мужской род. Убрали «Ты только начинаешь познавать нашу компанию».</t>
         </is>
@@ -4256,7 +4367,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr"/>
       <c r="J97" s="2" t="inlineStr"/>
-      <c r="K97" s="2" t="inlineStr">
+      <c r="N97" s="2" t="inlineStr">
         <is>
           <t>Кнопка «Со всем справился» → «Сложностей не было», без рода. Текст без «ты/вы».</t>
         </is>
@@ -4293,7 +4404,7 @@
       <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr"/>
       <c r="J98" s="2" t="inlineStr"/>
-      <c r="K98" s="2" t="inlineStr">
+      <c r="N98" s="2" t="inlineStr">
         <is>
           <t>Текст наш: в korsik_texts его нет.</t>
         </is>
@@ -4334,7 +4445,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr"/>
       <c r="J99" s="2" t="inlineStr"/>
-      <c r="K99" s="2" t="inlineStr">
+      <c r="N99" s="2" t="inlineStr">
         <is>
           <t>Кнопка «Не уверен» → «Пока сомневаюсь», без рода. Длинную кнопку «Готов озвучить причину в личной коммуникации с рекрутером» сократили до «Расскажу рекрутеру лично». Ответы «сомневаюсь» и «думаю об уходе» в нашем решении сразу уходят HR как красный флаг.</t>
         </is>
@@ -4371,7 +4482,7 @@
       <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr"/>
       <c r="J100" s="2" t="inlineStr"/>
-      <c r="K100" s="2" t="inlineStr"/>
+      <c r="N100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4404,7 +4515,7 @@
       <c r="H101" s="2" t="inlineStr"/>
       <c r="I101" s="2" t="inlineStr"/>
       <c r="J101" s="2" t="inlineStr"/>
-      <c r="K101" s="2" t="inlineStr"/>
+      <c r="N101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4437,7 +4548,7 @@
       <c r="H102" s="2" t="inlineStr"/>
       <c r="I102" s="2" t="inlineStr"/>
       <c r="J102" s="2" t="inlineStr"/>
-      <c r="K102" s="2" t="inlineStr"/>
+      <c r="N102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4466,7 +4577,7 @@
       <c r="H103" s="2" t="inlineStr"/>
       <c r="I103" s="2" t="inlineStr"/>
       <c r="J103" s="2" t="inlineStr"/>
-      <c r="K103" s="2" t="inlineStr">
+      <c r="N103" s="2" t="inlineStr">
         <is>
           <t>Как в строке 47: вопросы были на «вы», сделали две версии, логику «ниже 8 - уточнить» сохранили. Добавили вводную фразу, чтобы список не начинался без предупреждения. Девять оценок разбиты на шаги 64.1-64.9.</t>
         </is>
@@ -4503,7 +4614,7 @@
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr"/>
-      <c r="K104" s="2" t="inlineStr"/>
+      <c r="N104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -4536,7 +4647,7 @@
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr"/>
-      <c r="K105" s="2" t="inlineStr"/>
+      <c r="N105" s="2" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -4573,7 +4684,7 @@
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr"/>
-      <c r="K106" s="2" t="inlineStr"/>
+      <c r="N106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4606,7 +4717,7 @@
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr"/>
-      <c r="K107" s="2" t="inlineStr"/>
+      <c r="N107" s="2" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4639,7 +4750,7 @@
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr"/>
-      <c r="K108" s="2" t="inlineStr"/>
+      <c r="N108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -4672,7 +4783,7 @@
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr"/>
-      <c r="K109" s="2" t="inlineStr"/>
+      <c r="N109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4705,7 +4816,7 @@
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr"/>
-      <c r="K110" s="2" t="inlineStr"/>
+      <c r="N110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4738,7 +4849,7 @@
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr"/>
-      <c r="K111" s="2" t="inlineStr"/>
+      <c r="N111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4771,7 +4882,7 @@
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr"/>
-      <c r="K112" s="2" t="inlineStr"/>
+      <c r="N112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4804,7 +4915,7 @@
       <c r="H113" s="2" t="inlineStr"/>
       <c r="I113" s="2" t="inlineStr"/>
       <c r="J113" s="2" t="inlineStr"/>
-      <c r="K113" s="2" t="inlineStr">
+      <c r="N113" s="2" t="inlineStr">
         <is>
           <t>Было «Что порекомендуешь улучшить для более комфортной адаптации сотрудника?»: тяжело читается.</t>
         </is>
@@ -4841,7 +4952,7 @@
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr"/>
       <c r="J114" s="2" t="inlineStr"/>
-      <c r="K114" s="2" t="inlineStr">
+      <c r="N114" s="2" t="inlineStr">
         <is>
           <t>Без изменений по смыслу.</t>
         </is>
@@ -4878,7 +4989,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr"/>
       <c r="J115" s="2" t="inlineStr"/>
-      <c r="K115" s="2" t="inlineStr">
+      <c r="N115" s="2" t="inlineStr">
         <is>
           <t>Убрали из ссылки «?lang=en»: у русскоязычного пользователя страница должна открываться на русском. Ссылка стала кнопкой: в МАКС нельзя сделать ссылкой одно слово.</t>
         </is>
@@ -4927,7 +5038,7 @@
           <t>img_16.png</t>
         </is>
       </c>
-      <c r="K116" s="2" t="inlineStr">
+      <c r="N116" s="2" t="inlineStr">
         <is>
           <t>Сократили. Кнопку из шести эмодзи «😭😞😭😞🥺😞» заменили на одну.</t>
         </is>
@@ -4968,7 +5079,7 @@
           <t>img_13.png</t>
         </is>
       </c>
-      <c r="K117" s="2" t="inlineStr">
+      <c r="N117" s="2" t="inlineStr">
         <is>
           <t>Раньше бот так отвечал на любой вопрос. В новом решении это запасной ответ: сначала ИИ ищет ответ в базе знаний и отвечает со ссылкой на документ, и только если не нашёл - эта реплика. Не шаг по времени: так бот отвечает, когда передал вопрос HR.</t>
         </is>
@@ -5009,7 +5120,7 @@
           <t>img_12.png</t>
         </is>
       </c>
-      <c r="K118" s="2" t="inlineStr">
+      <c r="N118" s="2" t="inlineStr">
         <is>
           <t>Было «ты не прошел опрос»: звучит как упрёк и в мужском роде. Добавили кнопку, чтобы продолжить с того же места. Не шаг по времени: текст напоминания про вопрос без ответа. Кнопки «Продолжить опрос» нет.</t>
         </is>
@@ -5027,7 +5138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -5249,24 +5360,40 @@
       <c r="A37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Обязательный: «да» у шагов, которые получит даже новичок, открывший ссылку поздно (через неделю после того, как его завели, или после первого рабочего дня). Необязательные шаги, время которых прошло, такой новичок не получит, чтобы не завалить его сообщениями.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Кратко на «ты» и на «вы»: короткий текст обязательного шага для опоздавшего новичка. Пусто: уйдёт обычный текст. Такие шаги приходят в рабочее время его места работы, не больше трёх в день.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Комментарий: для людей, бот его не читает.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Строка 3 исходника не шаг: это описание бота, его ставят в профиль бота в МАКС (до 200 символов):</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>Я Корсик, помощник новичков Группы ПОЛИПЛАСТИК. Расскажу, как пройдут первые дни и месяцы, подскажу, где что найти, отвечу на вопросы по работе и позову HR, если нужен человек.</t>
         </is>

</xml_diff>

<commit_message>
newcomer checklist with nudges, answer ratings, leave risk, knowledge gaps, manager memos, lessons
</commit_message>
<xml_diff>
--- a/scenario/scenario.xlsx
+++ b/scenario/scenario.xlsx
@@ -56,7 +56,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -71,6 +71,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N118"/>
+  <dimension ref="A1:R118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -453,6 +456,10 @@
     <col width="45" customWidth="1" min="12" max="12"/>
     <col width="45" customWidth="1" min="13" max="13"/>
     <col width="55" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,6 +531,26 @@
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Комментарий</t>
+        </is>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
+        <is>
+          <t>Задача</t>
+        </is>
+      </c>
+      <c r="P1" s="6" t="inlineStr">
+        <is>
+          <t>Срок задачи</t>
+        </is>
+      </c>
+      <c r="Q1" s="6" t="inlineStr">
+        <is>
+          <t>Проверка</t>
+        </is>
+      </c>
+      <c r="R1" s="6" t="inlineStr">
+        <is>
+          <t>Руководителю</t>
         </is>
       </c>
     </row>
@@ -762,6 +789,21 @@
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Было «чтобы ты пришел подготовленный»: мужской род и канцелярит. Добавили, что делать, если документа нет. Список в колонке J: без «Вашего», с единым оформлением. Список документов из колонки J добавлен в конец текста.</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>Собрать документы для оформления</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>-1д 18:00</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>Все документы для оформления собраны?</t>
         </is>
       </c>
     </row>
@@ -834,6 +876,21 @@
           <t>Как в строке 9. Для GTP в списке есть фото 3×4, для GrPP и Luzhniki - нет. Уточнить у HR, так и задумано или фото нужно всем. Список документов из колонки J добавлен в конец текста.</t>
         </is>
       </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>Собрать документы для оформления</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>-1д 18:00</t>
+        </is>
+      </c>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Все документы для оформления собраны?</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1068,6 +1125,15 @@
       <c r="N13" s="2" t="inlineStr">
         <is>
           <t>Кнопка «Готов/Готова» → «Всё готово», без рода. Убрали шутку «я сам через это проходил, когда меня создавали»: она обесценивает волнение. Добавили, что боту можно писать. Время в исходнике не указано, взяли 10:00. Ответ сохраняется как опрос.</t>
+        </is>
+      </c>
+      <c r="R13" s="4" t="inlineStr">
+        <is>
+          <t>Завтра у вас выходит новый сотрудник: {новичок}. Подсказки на старте:
+• проверьте, что рабочее место и доступы будут готовы к утру;
+• встретьте лично и познакомьте с командой;
+• назначьте наставника, к которому можно подойти с любым вопросом;
+• в первые три дня обсудите адаптационный план.</t>
         </is>
       </c>
     </row>
@@ -1294,6 +1360,21 @@
           <t>Сократили. Убрали общие фразы («вносить свой вклад в наше общее дело», «создать комфортные условия»), оставили главное: спрашивать можно и нужно.</t>
         </is>
       </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>Пройти обучение в приложении: правила распорядка и охрана труда</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>р5 17:00</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>Получилось пройти обучение в приложении бота?</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2242,6 +2323,29 @@
 Правка движка: убрали «Вот он.», плана во вложении пока нет.</t>
         </is>
       </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>Обсудить адаптационный план с руководителем</t>
+        </is>
+      </c>
+      <c r="P41" s="4" t="inlineStr">
+        <is>
+          <t>р5 17:00</t>
+        </is>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>Получилось обсудить адаптационный план с руководителем?</t>
+        </is>
+      </c>
+      <c r="R41" s="4" t="inlineStr">
+        <is>
+          <t>Сегодня {новичок} получает адаптационный план. Памятка к разговору:
+• пройдитесь по задачам испытательного срока и срокам;
+• договоритесь, как и когда давать обратную связь;
+• спросите, что непонятно и чего не хватает для работы.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3388,6 +3492,26 @@
       <c r="N73" s="2" t="inlineStr">
         <is>
           <t>Было «закреплённый за тобой Сотрудник Отдела по подбору и адаптации персонала»: канцелярит и лишние заглавные. Время в исходнике не указано, взяли 10:00.</t>
+        </is>
+      </c>
+      <c r="O73" s="4" t="inlineStr">
+        <is>
+          <t>Встреча с менеджером по подбору по адаптационному плану</t>
+        </is>
+      </c>
+      <c r="P73" s="4" t="inlineStr">
+        <is>
+          <t>м1+17д 17:00</t>
+        </is>
+      </c>
+      <c r="Q73" s="4" t="inlineStr">
+        <is>
+          <t>Встреча с менеджером по подбору уже прошла?</t>
+        </is>
+      </c>
+      <c r="R73" s="4" t="inlineStr">
+        <is>
+          <t>Через 2–3 дня у {новичок} встреча с менеджером по подбору: обсуждают, как идёт адаптационный план. Памятка: посмотрите, что из плана сделано, и расскажите менеджеру, где новичку нужна помощь.</t>
         </is>
       </c>
     </row>
@@ -4333,6 +4457,14 @@
       <c r="N96" s="2" t="inlineStr">
         <is>
           <t>Было «Дорогой Х»: мужской род. Убрали «Ты только начинаешь познавать нашу компанию».</t>
+        </is>
+      </c>
+      <c r="R96" s="4" t="inlineStr">
+        <is>
+          <t>У {новичок} заканчивается испытательный срок. Памятка к итоговой встрече:
+• что удалось и что нет из адаптационного плана;
+• как новичок видит свою работу дальше;
+• решение по испытательному сроку и следующие цели.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5498,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
@@ -5374,7 +5505,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>

</xml_diff>